<commit_message>
Rebuild from the Google files (2026-10-23)
Fresh downloads of the framework Doc, the game text Sheet and the
commons-comma matrix and packet: three tries to solve the case, no
follow-up bonus, the revised Rules of the game, and the sidebar's
"HEAR Framework Guide" link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J8R4SET6LminzKA26BGVqh
</commit_message>
<xml_diff>
--- a/engine/HEARsay game text.xlsx
+++ b/engine/HEARsay game text.xlsx
@@ -13,30 +13,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="266">
   <si>
     <t>Sheet</t>
+  </si>
+  <si>
+    <t>Engine passage</t>
   </si>
   <si>
     <t>Key</t>
   </si>
   <si>
-    <t>Engine passage</t>
+    <t>Framework name</t>
   </si>
   <si>
     <t>What it holds</t>
   </si>
   <si>
-    <t>Framework name</t>
-  </si>
-  <si>
     <t>Framework section</t>
   </si>
   <si>
-    <t>Notes</t>
+    <t>Text</t>
   </si>
   <si>
-    <t>Text</t>
+    <t>Notes</t>
   </si>
   <si>
     <t>Start</t>
@@ -48,13 +48,13 @@
     <t>Placeholders</t>
   </si>
   <si>
+    <t>3.1</t>
+  </si>
+  <si>
     <t>menu.map</t>
   </si>
   <si>
     <t>Sidebar</t>
-  </si>
-  <si>
-    <t>3.1</t>
   </si>
   <si>
     <t>Campus map</t>
@@ -69,37 +69,31 @@
     <t>the Hook</t>
   </si>
   <si>
-    <t>label</t>
-  </si>
-  <si>
     <t>3.2</t>
   </si>
   <si>
     <t>Shown after the introduction, then the Map. The scenario's Hook text comes from the Response Matrix (Passages sheet, 'the Hook').</t>
   </si>
   <si>
+    <t>Rules</t>
+  </si>
+  <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>Introduction, part 2: the rules. Shown once after Start; then the Hook.</t>
+  </si>
+  <si>
     <t>menu.evidence</t>
   </si>
   <si>
-    <t>Rules</t>
+    <t>Rules Summary</t>
   </si>
   <si>
     <t>Evidence board</t>
   </si>
   <si>
-    <t>Introduction, part 2: the rules. Shown once after Start; then the Hook.</t>
-  </si>
-  <si>
-    <t>menu.case_file</t>
-  </si>
-  <si>
-    <t>Rules Summary</t>
-  </si>
-  <si>
     <t>A slide with these rules</t>
-  </si>
-  <si>
-    <t>Case file</t>
   </si>
   <si>
     <t>The same rules, always available from the sidebar.</t>
@@ -108,40 +102,64 @@
     <t>HEAR Guide</t>
   </si>
   <si>
-    <t>menu.hear</t>
+    <t>menu.case_file</t>
   </si>
   <si>
     <t>A slide with a quick summary of the HEAR framework</t>
   </si>
   <si>
-    <t>HEAR guide</t>
+    <t>Case file</t>
   </si>
   <si>
     <t>Always available from the sidebar.</t>
   </si>
   <si>
-    <t>The game's own text: everything the player reads that is the same in every scenario (rules, the HEAR guide, headings, buttons, prompts), and the framework's numbers. Scenario text lives in each scenario's Response Matrix. The build checks this workbook against an export of the framework Google Doc ('HEARsay mysteries'), the way it checks a matrix against its packet.</t>
+    <t>menu.hear</t>
   </si>
   <si>
     <t>Map</t>
   </si>
   <si>
-    <t>menu.rules</t>
+    <t>3.3</t>
   </si>
   <si>
-    <t>3.3</t>
+    <t>HEAR Framework Guide</t>
   </si>
   <si>
     <t>Interview</t>
   </si>
   <si>
+    <t>The game's own text: everything the player reads that is the same in every scenario (rules, the HEAR guide, headings, buttons, prompts), and the framework's numbers. Scenario text lives in each scenario's Response Matrix. The build checks this workbook against an export of the framework Google Doc ('HEARsay mysteries'), the way it checks a matrix against its packet.</t>
+  </si>
+  <si>
+    <t>Answer</t>
+  </si>
+  <si>
+    <t>Follow-up</t>
+  </si>
+  <si>
+    <t>menu.rules</t>
+  </si>
+  <si>
+    <t>3.3.1</t>
+  </si>
+  <si>
+    <t>Follow-up Result</t>
+  </si>
+  <si>
     <t>sidebar.questions_left</t>
+  </si>
+  <si>
+    <t>Engine addition: shows the Major Clue and the explanation, or the walk-away.</t>
   </si>
   <si>
     <t>Questions left: **{left}**</t>
   </si>
   <si>
-    <t>Answer</t>
+    <t>Evidence Board</t>
+  </si>
+  <si>
+    <t>4</t>
   </si>
   <si>
     <t>left</t>
@@ -150,49 +168,67 @@
     <t>sidebar.submitted</t>
   </si>
   <si>
+    <t>Case File</t>
+  </si>
+  <si>
     <t>Case submitted</t>
   </si>
   <si>
-    <t>Follow-up</t>
+    <t>Engine addition: the mystery and the Hook's brief and controversy, always available from the sidebar.</t>
   </si>
   <si>
-    <t>3.3.1</t>
+    <t>Passages</t>
+  </si>
+  <si>
+    <t>Submission</t>
+  </si>
+  <si>
+    <t>3.4</t>
+  </si>
+  <si>
+    <t>sidebar.tries_left</t>
+  </si>
+  <si>
+    <t>Each screen of the game, with the name the framework gives it. The build stops if a passage the framework lists (section 4, 'Passages text') has no screen, or if a framework name here does not appear in the framework.</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Tries left: **{left}**</t>
+  </si>
+  <si>
+    <t>The verdict and the scenario's ending text for that verdict.</t>
   </si>
   <si>
     <t>status.questions_left</t>
   </si>
   <si>
-    <t>Passages</t>
-  </si>
-  <si>
-    <t>Follow-up Result</t>
+    <t>Ranking</t>
   </si>
   <si>
     <t>Questions left: **{left}** / {budget}</t>
   </si>
   <si>
-    <t>Each screen of the game, with the name the framework gives it. The build stops if a passage the framework lists (section 4, 'Passages text') has no screen, or if a framework name here does not appear in the framework.</t>
-  </si>
-  <si>
-    <t>Engine addition: shows the Major Clue and the explanation, or the walk-away.</t>
+    <t>ranking</t>
   </si>
   <si>
     <t>status.hear_aria</t>
   </si>
   <si>
-    <t>Evidence Board</t>
+    <t>Ending</t>
+  </si>
+  <si>
+    <t>ending</t>
   </si>
   <si>
     <t>HEAR letters earned: {n} of 4</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>n</t>
   </si>
   <si>
-    <t>Case File</t>
+    <t>The debrief: scores, the solution, the full ending, the Major Clues and the red-herring sets.</t>
   </si>
   <si>
     <t>common.portrait_alt</t>
@@ -201,22 +237,19 @@
     <t>Portrait of {name}</t>
   </si>
   <si>
-    <t>Engine addition: the mystery and the Hook's brief and controversy, always available from the sidebar.</t>
-  </si>
-  <si>
     <t>name</t>
   </si>
   <si>
-    <t>Submission</t>
+    <t>Engine addition: the menu, the question counter and the HEAR letters.</t>
   </si>
   <si>
     <t>common.map_alt</t>
   </si>
   <si>
-    <t>3.4</t>
+    <t>Newspaper</t>
   </si>
   <si>
-    <t>Result</t>
+    <t>One row per piece of text. Check = verbatim: the text must appear word for word in the framework. Check = paraphrase: it restates the framework section named, which must exist. Check = label: engine wording the framework does not cover. {curly} words are filled in by the game; the ones every text can use are listed below, others in the Placeholders column. **Double asterisks** make words bold. Rules rows (rules.1, rules.2 …) are shown in number order, so rows can be added or removed. Spaces at the start or end of a cell are ignored.</t>
   </si>
   <si>
     <t>common.solve</t>
@@ -225,34 +258,16 @@
     <t>Solve the case</t>
   </si>
   <si>
-    <t>One row per piece of text. Check = verbatim: the text must appear word for word in the framework. Check = paraphrase: it restates the framework section named, which must exist. Check = label: engine wording the framework does not cover. {curly} words are filled in by the game; the ones every text can use are listed below, others in the Placeholders column. **Double asterisks** make words bold. Rules rows (rules.1, rules.2 …) are shown in number order, so rows can be added or removed. Spaces at the start or end of a cell are ignored.</t>
-  </si>
-  <si>
-    <t>The verdict and the scenario's ending text for that verdict.</t>
-  </si>
-  <si>
-    <t>Ranking</t>
+    <t>Engine addition: the scenario's newspaper article (the packet's 'Newspaper article' tab), shown once between the Rules and the Hook and always available from the sidebar. Only in scenarios whose packet has that tab.</t>
   </si>
   <si>
     <t>common.submit_now</t>
   </si>
   <si>
-    <t>ranking</t>
-  </si>
-  <si>
     <t>Submit your solution</t>
   </si>
   <si>
-    <t>Ending</t>
-  </si>
-  <si>
-    <t>ending</t>
-  </si>
-  <si>
     <t>common.back_to_map</t>
-  </si>
-  <si>
-    <t>The debrief: scores, the solution, the full ending, the Major Clues and the red-herring sets.</t>
   </si>
   <si>
     <t>Back to map</t>
@@ -261,34 +276,16 @@
     <t>common.return</t>
   </si>
   <si>
-    <t>Engine addition: the menu, the question counter and the HEAR letters.</t>
-  </si>
-  <si>
     <t>Return</t>
   </si>
   <si>
     <t>Facts</t>
   </si>
   <si>
-    <t>Newspaper</t>
+    <t>common.evidence</t>
   </si>
   <si>
     <t>The framework's numbers. Framework wording must appear in the framework and contain the value; the build checks every scenario against these. A fact with no framework wording is an engine choice the framework does not state yet, and the build lists it as a note.</t>
-  </si>
-  <si>
-    <t>Engine addition: the scenario's newspaper article (the packet's 'Newspaper article' tab), shown once between the Rules and the Hook and always available from the sidebar. Only in scenarios whose packet has that tab.</t>
-  </si>
-  <si>
-    <t>Every text can use {budget} {n_witnesses} {n_questions} {n_major} {bonus} {rank_exact} {rank_near} {ccc} {title}.</t>
-  </si>
-  <si>
-    <t>Source of truth</t>
-  </si>
-  <si>
-    <t>This Google Sheet is the source of truth for the game text. Edit it here. Each build downloads it into the repository as engine/HEARsay game text.xlsx, a snapshot that nobody edits by hand, and commits the snapshot with the rebuilt games.</t>
-  </si>
-  <si>
-    <t>common.evidence</t>
   </si>
   <si>
     <t>common.map</t>
@@ -315,6 +312,9 @@
     <t>hook.assignment</t>
   </si>
   <si>
+    <t>Every text can use {budget} {n_witnesses} {n_questions} {n_major} {rank_exact} {rank_near} {ccc} {title}.</t>
+  </si>
+  <si>
     <t>Your assignment</t>
   </si>
   <si>
@@ -339,7 +339,13 @@
     <t>rules.next</t>
   </si>
   <si>
+    <t>Source of truth</t>
+  </si>
+  <si>
     <t>Begin the case</t>
+  </si>
+  <si>
+    <t>This Google Sheet is the source of truth for the game text. Edit it here. Each build downloads it into the repository as engine/HEARsay game text.xlsx, a snapshot that nobody edits by hand, and commits the snapshot with the rebuilt games.</t>
   </si>
   <si>
     <t>case.title</t>
@@ -543,15 +549,6 @@
     <t>receptive follow-up</t>
   </si>
   <si>
-    <t>evidence.bonus</t>
-  </si>
-  <si>
-    <t>Bonus points so far: {points}</t>
-  </si>
-  <si>
-    <t>points</t>
-  </si>
-  <si>
     <t>submit.title</t>
   </si>
   <si>
@@ -579,6 +576,27 @@
     <t>Keep investigating</t>
   </si>
   <si>
+    <t>submit.wrong</t>
+  </si>
+  <si>
+    <t>That isn't the solution. Tries left: **{left}**</t>
+  </si>
+  <si>
+    <t>submit.tried</t>
+  </si>
+  <si>
+    <t>Already tried: {who} and “{where}”</t>
+  </si>
+  <si>
+    <t>who where</t>
+  </si>
+  <si>
+    <t>submit.repeat</t>
+  </si>
+  <si>
+    <t>You already tried that answer.</t>
+  </si>
+  <si>
     <t>result.correct</t>
   </si>
   <si>
@@ -601,9 +619,6 @@
   </si>
   <si>
     <t>You named {who} and “{where}”.</t>
-  </si>
-  <si>
-    <t>who where</t>
   </si>
   <si>
     <t>result.one_more</t>
@@ -684,16 +699,28 @@
     <t>score</t>
   </si>
   <si>
-    <t>ending.bonus</t>
-  </si>
-  <si>
-    <t>Follow-up bonus: **{points}**</t>
-  </si>
-  <si>
     <t>ending.used</t>
   </si>
   <si>
     <t>Questions used: **{n} of {budget}**</t>
+  </si>
+  <si>
+    <t>ending.tries</t>
+  </si>
+  <si>
+    <t>Tries used: **{n} of {total}**</t>
+  </si>
+  <si>
+    <t>n total</t>
+  </si>
+  <si>
+    <t>ending.solve_points</t>
+  </si>
+  <si>
+    <t>Solving points: **{points} of {total}**</t>
+  </si>
+  <si>
+    <t>points total</t>
   </si>
   <si>
     <t>ending.table_title</t>
@@ -730,9 +757,6 @@
   </si>
   <si>
     <t>{n} of {total}</t>
-  </si>
-  <si>
-    <t>n total</t>
   </si>
   <si>
     <t>ending.solution</t>
@@ -833,11 +857,11 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf quotePrefix="1" borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -1082,37 +1106,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
-      <c r="V1" s="2"/>
-      <c r="W1" s="2"/>
-      <c r="X1" s="2"/>
-      <c r="Y1" s="2"/>
-      <c r="Z1" s="2"/>
+        <v>4</v>
+      </c>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="3"/>
+      <c r="T1" s="3"/>
+      <c r="U1" s="3"/>
+      <c r="V1" s="3"/>
+      <c r="W1" s="3"/>
+      <c r="X1" s="3"/>
+      <c r="Y1" s="3"/>
+      <c r="Z1" s="3"/>
     </row>
     <row r="2">
       <c r="A2" s="5"/>
-      <c r="B2" s="3" t="s">
-        <v>35</v>
+      <c r="B2" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -1140,11 +1164,11 @@
       <c r="Z2" s="5"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>52</v>
+      <c r="A3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -1172,11 +1196,11 @@
       <c r="Z3" s="5"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>70</v>
+      <c r="A4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -1204,11 +1228,11 @@
       <c r="Z4" s="5"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>86</v>
+      <c r="A5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -1236,11 +1260,11 @@
       <c r="Z5" s="5"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>88</v>
+      <c r="B6" s="6" t="s">
+        <v>99</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -1268,11 +1292,11 @@
       <c r="Z6" s="5"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>90</v>
+      <c r="A7" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>110</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -29123,240 +29147,240 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="3" t="s">
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
+      <c r="B4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="3" t="s">
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>29</v>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="3" t="s">
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>36</v>
+      <c r="B7" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D7" s="5"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="5"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="5"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="s">
+      <c r="C9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="5"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C10" s="3" t="s">
+      <c r="D11" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="5"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>55</v>
-      </c>
       <c r="C12" s="4" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D12" s="5"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="s">
-        <v>59</v>
+      <c r="A13" s="2" t="s">
+        <v>51</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
-      <c r="D13" s="3" t="s">
-        <v>62</v>
+      <c r="D13" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>64</v>
+      <c r="A14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>55</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="D14" s="5"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="5"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D15" s="3" t="s">
+      <c r="B17" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D16" s="5"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
     <row r="18">
-      <c r="A18" s="3" t="s">
-        <v>12</v>
+      <c r="A18" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
-      <c r="D18" s="3" t="s">
-        <v>82</v>
+      <c r="D18" s="2" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
       <c r="D19" s="6" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20">
@@ -29511,13 +29535,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>5</v>
@@ -29530,1635 +29554,1673 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D2" s="5"/>
-      <c r="E2" s="3" t="s">
-        <v>18</v>
+      <c r="E2" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="F2" s="5"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="F3" s="5"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="5"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="5"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="5"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15" s="5"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" s="5"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="5"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="s">
+      <c r="D18" s="5"/>
+      <c r="E18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="5"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19" s="5"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F21" s="5"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D22" s="5"/>
+      <c r="E22" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" s="5"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="5"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D24" s="5"/>
+      <c r="E24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" s="5"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25" s="5"/>
+      <c r="E25" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F25" s="5"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D26" s="5"/>
+      <c r="E26" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" s="5"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D27" s="5"/>
+      <c r="E27" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F27" s="5"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="5"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="s">
+      <c r="D28" s="5"/>
+      <c r="E28" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" s="5"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D29" s="5"/>
+      <c r="E29" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F29" s="5"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D30" s="5"/>
+      <c r="E30" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" s="5"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D31" s="5"/>
+      <c r="E31" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F31" s="5"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="5"/>
+      <c r="E32" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F32" s="5"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F33" s="5"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D35" s="5"/>
+      <c r="E35" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" s="5"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F36" s="5"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D37" s="5"/>
+      <c r="E37" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F37" s="5"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="5"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="s">
+      <c r="C38" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D38" s="5"/>
+      <c r="E38" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D39" s="5"/>
+      <c r="E39" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D40" s="5"/>
+      <c r="E40" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D41" s="5"/>
+      <c r="E41" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D42" s="5"/>
+      <c r="E42" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="3" t="s">
+      <c r="C43" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D43" s="5"/>
+      <c r="E43" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D44" s="5"/>
+      <c r="E44" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F44" s="5"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="5"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="3" t="s">
+      <c r="C45" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D45" s="5"/>
+      <c r="E45" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" s="3" t="s">
+      <c r="C46" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D46" s="5"/>
+      <c r="E46" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D47" s="5"/>
+      <c r="E47" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F47" s="5"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D48" s="5"/>
+      <c r="E48" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D49" s="5"/>
+      <c r="E49" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F49" s="5"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D50" s="5"/>
+      <c r="E50" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F50" s="5"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D51" s="5"/>
+      <c r="E51" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F51" s="5"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D52" s="5"/>
+      <c r="E52" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F52" s="5"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D53" s="5"/>
+      <c r="E53" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F53" s="5"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D54" s="5"/>
+      <c r="E54" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F54" s="5"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D55" s="5"/>
+      <c r="E55" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D56" s="5"/>
+      <c r="E56" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F56" s="5"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D57" s="5"/>
+      <c r="E57" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D58" s="5"/>
+      <c r="E58" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F58" s="5"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D59" s="5"/>
+      <c r="E59" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F59" s="5"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D60" s="5"/>
+      <c r="E60" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F60" s="5"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D61" s="5"/>
+      <c r="E61" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F61" s="5"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D62" s="5"/>
+      <c r="E62" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F62" s="5"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D63" s="5"/>
+      <c r="E63" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F63" s="5"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D64" s="5"/>
+      <c r="E64" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F64" s="5"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D65" s="5"/>
+      <c r="E65" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F65" s="5"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D66" s="5"/>
+      <c r="E66" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="D67" s="5"/>
+      <c r="E67" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="D68" s="5"/>
+      <c r="E68" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F68" s="5"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D69" s="5"/>
+      <c r="E69" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F69" s="5"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D70" s="5"/>
+      <c r="E70" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F70" s="5"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D71" s="5"/>
+      <c r="E71" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F71" s="5"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D72" s="5"/>
+      <c r="E72" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D73" s="5"/>
+      <c r="E73" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F73" s="5"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D74" s="5"/>
+      <c r="E74" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F74" s="5"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="D75" s="5"/>
+      <c r="E75" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F75" s="5"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B76" s="2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F12" s="5"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F13" s="5"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F14" s="5"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F15" s="5"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F16" s="5"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D17" s="5"/>
-      <c r="E17" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F17" s="5"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F18" s="5"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D19" s="5"/>
-      <c r="E19" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F19" s="5"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="D20" s="5"/>
-      <c r="E20" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F20" s="5"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="D21" s="5"/>
-      <c r="E21" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F21" s="5"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="D22" s="5"/>
-      <c r="E22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F22" s="5"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="D23" s="5"/>
-      <c r="E23" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F23" s="5"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D24" s="5"/>
-      <c r="E24" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F24" s="5"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="D25" s="5"/>
-      <c r="E25" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F25" s="5"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="D26" s="5"/>
-      <c r="E26" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F26" s="5"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D27" s="5"/>
-      <c r="E27" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F27" s="5"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="D28" s="5"/>
-      <c r="E28" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F28" s="5"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="D29" s="5"/>
-      <c r="E29" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F29" s="5"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D30" s="5"/>
-      <c r="E30" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F30" s="5"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D31" s="5"/>
-      <c r="E31" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F31" s="5"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D32" s="5"/>
-      <c r="E32" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F32" s="5"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="D33" s="5"/>
-      <c r="E33" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="D34" s="5"/>
-      <c r="E34" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F34" s="5"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="D35" s="5"/>
-      <c r="E35" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F35" s="5"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="D36" s="5"/>
-      <c r="E36" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F36" s="5"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="D37" s="5"/>
-      <c r="E37" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D38" s="5"/>
-      <c r="E38" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F38" s="3" t="s">
+      <c r="C76" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D76" s="5"/>
+      <c r="E76" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F76" s="5"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B77" s="2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D39" s="5"/>
-      <c r="E39" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D40" s="5"/>
-      <c r="E40" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D41" s="5"/>
-      <c r="E41" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D42" s="5"/>
-      <c r="E42" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="D43" s="5"/>
-      <c r="E43" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F43" s="5"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="D44" s="5"/>
-      <c r="E44" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="D45" s="5"/>
-      <c r="E45" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F45" s="3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="D46" s="5"/>
-      <c r="E46" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F46" s="5"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="D47" s="5"/>
-      <c r="E47" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F47" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="D48" s="5"/>
-      <c r="E48" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F48" s="5"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D49" s="5"/>
-      <c r="E49" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F49" s="5"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="D50" s="5"/>
-      <c r="E50" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F50" s="5"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="D51" s="5"/>
-      <c r="E51" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F51" s="5"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C52" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="D52" s="5"/>
-      <c r="E52" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F52" s="5"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="D53" s="5"/>
-      <c r="E53" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F53" s="5"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D54" s="5"/>
-      <c r="E54" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F54" s="3" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D55" s="5"/>
-      <c r="E55" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F55" s="5"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="D56" s="5"/>
-      <c r="E56" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="D57" s="5"/>
-      <c r="E57" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F57" s="5"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="D58" s="5"/>
-      <c r="E58" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F58" s="5"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="D59" s="5"/>
-      <c r="E59" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F59" s="5"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="D60" s="5"/>
-      <c r="E60" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F60" s="3" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D61" s="5"/>
-      <c r="E61" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F61" s="5"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="D62" s="5"/>
-      <c r="E62" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F62" s="5"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="D63" s="5"/>
-      <c r="E63" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F63" s="5"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="D64" s="5"/>
-      <c r="E64" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F64" s="5"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="D65" s="5"/>
-      <c r="E65" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F65" s="5"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="B66" s="3" t="s">
+      <c r="C77" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D77" s="5"/>
+      <c r="E77" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F77" s="5"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B78" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C66" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="D66" s="5"/>
-      <c r="E66" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F66" s="5"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="B67" s="3" t="s">
+      <c r="C78" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D78" s="5"/>
+      <c r="E78" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F78" s="5"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B79" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C67" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="D67" s="5"/>
-      <c r="E67" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F67" s="5"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="B68" s="3" t="s">
+      <c r="C79" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D79" s="5"/>
+      <c r="E79" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B80" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C68" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="D68" s="5"/>
-      <c r="E68" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F68" s="5"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="B69" s="3" t="s">
+      <c r="C80" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="D80" s="5"/>
+      <c r="E80" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F80" s="5"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B81" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C69" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="D69" s="5"/>
-      <c r="E69" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="B70" s="3" t="s">
+      <c r="C81" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="D81" s="5"/>
+      <c r="E81" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F81" s="5"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B82" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C70" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="D70" s="5"/>
-      <c r="E70" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F70" s="5"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="B71" s="3" t="s">
+      <c r="C82" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D82" s="5"/>
+      <c r="E82" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F82" s="5"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B83" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C71" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="D71" s="5"/>
-      <c r="E71" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F71" s="5"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="B72" s="3" t="s">
+      <c r="C83" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="D83" s="5"/>
+      <c r="E83" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B84" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C72" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="D72" s="5"/>
-      <c r="E72" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F72" s="5"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="D73" s="5"/>
-      <c r="E73" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F73" s="5"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C74" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="D74" s="5"/>
-      <c r="E74" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F74" s="5"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C75" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="D75" s="5"/>
-      <c r="E75" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F75" s="5"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="D76" s="5"/>
-      <c r="E76" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F76" s="3" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="D77" s="5"/>
-      <c r="E77" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F77" s="5"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="D78" s="5"/>
-      <c r="E78" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F78" s="5"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C79" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="D79" s="5"/>
-      <c r="E79" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F79" s="5"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C80" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="D80" s="5"/>
-      <c r="E80" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F80" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C81" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="D81" s="5"/>
-      <c r="E81" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F81" s="3" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="B82" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C82" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="D82" s="5"/>
-      <c r="E82" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F82" s="3" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C83" s="3" t="s">
+      <c r="C84" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="D83" s="5"/>
-      <c r="E83" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F83" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="3" t="s">
+      <c r="D84" s="5"/>
+      <c r="E84" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F84" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B84" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C84" s="3" t="s">
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="D84" s="5"/>
-      <c r="E84" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F84" s="5"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="3" t="s">
+      <c r="B85" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C85" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="B85" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C85" s="3" t="s">
+      <c r="D85" s="5"/>
+      <c r="E85" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="D85" s="5"/>
-      <c r="E85" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F85" s="5"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="3" t="s">
+      <c r="B86" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C86" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="B86" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C86" s="3" t="s">
+      <c r="D86" s="5"/>
+      <c r="E86" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F86" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="D86" s="5"/>
-      <c r="E86" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F86" s="5"/>
     </row>
     <row r="87">
-      <c r="A87" s="3" t="s">
+      <c r="A87" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="B87" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C87" s="3" t="s">
+      <c r="B87" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C87" s="6" t="s">
         <v>234</v>
       </c>
       <c r="D87" s="5"/>
-      <c r="E87" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F87" s="5"/>
+      <c r="E87" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F87" s="6" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="B88" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C88" s="3" t="s">
+      <c r="A88" s="2" t="s">
         <v>236</v>
       </c>
+      <c r="B88" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>237</v>
+      </c>
       <c r="D88" s="5"/>
-      <c r="E88" s="3" t="s">
-        <v>18</v>
+      <c r="E88" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="F88" s="5"/>
     </row>
     <row r="89">
-      <c r="A89" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="B89" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C89" s="3" t="s">
+      <c r="A89" s="2" t="s">
         <v>238</v>
       </c>
+      <c r="B89" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>239</v>
+      </c>
       <c r="D89" s="5"/>
-      <c r="E89" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F89" s="3" t="s">
-        <v>239</v>
-      </c>
+      <c r="E89" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F89" s="5"/>
     </row>
     <row r="90">
-      <c r="A90" s="3" t="s">
+      <c r="A90" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="B90" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C90" s="3" t="s">
+      <c r="B90" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C90" s="2" t="s">
         <v>241</v>
       </c>
       <c r="D90" s="5"/>
-      <c r="E90" s="3" t="s">
-        <v>18</v>
+      <c r="E90" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="F90" s="5"/>
     </row>
     <row r="91">
-      <c r="A91" s="3" t="s">
+      <c r="A91" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="B91" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C91" s="3" t="s">
+      <c r="B91" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C91" s="2" t="s">
         <v>243</v>
       </c>
       <c r="D91" s="5"/>
-      <c r="E91" s="3" t="s">
-        <v>18</v>
+      <c r="E91" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="F91" s="5"/>
     </row>
     <row r="92">
-      <c r="A92" s="3" t="s">
+      <c r="A92" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="B92" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C92" s="3" t="s">
+      <c r="B92" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C92" s="2" t="s">
         <v>245</v>
       </c>
       <c r="D92" s="5"/>
-      <c r="E92" s="3" t="s">
-        <v>18</v>
+      <c r="E92" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="F92" s="5"/>
     </row>
     <row r="93">
-      <c r="A93" s="3" t="s">
+      <c r="A93" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B93" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C93" s="3" t="s">
+      <c r="B93" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C93" s="2" t="s">
         <v>247</v>
       </c>
       <c r="D93" s="5"/>
-      <c r="E93" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F93" s="5"/>
+      <c r="E93" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="3" t="s">
+      <c r="A94" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="B94" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C94" s="3" t="s">
+      <c r="B94" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C94" s="2" t="s">
         <v>249</v>
       </c>
       <c r="D94" s="5"/>
-      <c r="E94" s="3" t="s">
-        <v>18</v>
+      <c r="E94" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="F94" s="5"/>
     </row>
     <row r="95">
-      <c r="A95" s="6" t="s">
+      <c r="A95" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="B95" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C95" s="6" t="s">
+      <c r="B95" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C95" s="2" t="s">
         <v>251</v>
       </c>
       <c r="D95" s="5"/>
-      <c r="E95" s="6" t="s">
-        <v>18</v>
+      <c r="E95" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="F95" s="5"/>
     </row>
     <row r="96">
-      <c r="A96" s="6" t="s">
+      <c r="A96" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B96" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="C96" s="6" t="s">
+      <c r="B96" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C96" s="2" t="s">
         <v>253</v>
       </c>
       <c r="D96" s="5"/>
-      <c r="E96" s="6" t="s">
-        <v>18</v>
+      <c r="E96" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="F96" s="5"/>
     </row>
     <row r="97">
-      <c r="A97" s="6" t="s">
+      <c r="A97" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="B97" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="C97" s="6" t="s">
+      <c r="B97" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C97" s="2" t="s">
         <v>255</v>
       </c>
       <c r="D97" s="5"/>
-      <c r="E97" s="6" t="s">
-        <v>18</v>
+      <c r="E97" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="F97" s="5"/>
     </row>
     <row r="98">
-      <c r="A98" s="6" t="s">
+      <c r="A98" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="B98" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="C98" s="6" t="s">
+      <c r="B98" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C98" s="2" t="s">
         <v>257</v>
       </c>
       <c r="D98" s="5"/>
-      <c r="E98" s="6" t="s">
-        <v>18</v>
+      <c r="E98" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="F98" s="5"/>
     </row>
     <row r="99">
-      <c r="A99" s="5"/>
-      <c r="B99" s="5"/>
-      <c r="C99" s="5"/>
+      <c r="A99" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>259</v>
+      </c>
       <c r="D99" s="5"/>
-      <c r="E99" s="5"/>
+      <c r="E99" s="6" t="s">
+        <v>21</v>
+      </c>
       <c r="F99" s="5"/>
     </row>
     <row r="100">
-      <c r="A100" s="5"/>
-      <c r="B100" s="5"/>
-      <c r="C100" s="5"/>
+      <c r="A100" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>261</v>
+      </c>
       <c r="D100" s="5"/>
-      <c r="E100" s="5"/>
+      <c r="E100" s="6" t="s">
+        <v>21</v>
+      </c>
       <c r="F100" s="5"/>
     </row>
     <row r="101">
-      <c r="A101" s="5"/>
-      <c r="B101" s="5"/>
-      <c r="C101" s="5"/>
+      <c r="A101" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>263</v>
+      </c>
       <c r="D101" s="5"/>
-      <c r="E101" s="5"/>
+      <c r="E101" s="6" t="s">
+        <v>21</v>
+      </c>
       <c r="F101" s="5"/>
     </row>
     <row r="102">
-      <c r="A102" s="5"/>
-      <c r="B102" s="5"/>
-      <c r="C102" s="5"/>
+      <c r="A102" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>265</v>
+      </c>
       <c r="D102" s="5"/>
-      <c r="E102" s="5"/>
+      <c r="E102" s="6" t="s">
+        <v>21</v>
+      </c>
       <c r="F102" s="5"/>
     </row>
     <row r="103">
@@ -31729,6 +31791,38 @@
       <c r="E173" s="5"/>
       <c r="F173" s="5"/>
     </row>
+    <row r="174">
+      <c r="A174" s="5"/>
+      <c r="B174" s="5"/>
+      <c r="C174" s="5"/>
+      <c r="D174" s="5"/>
+      <c r="E174" s="5"/>
+      <c r="F174" s="5"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="5"/>
+      <c r="B175" s="5"/>
+      <c r="C175" s="5"/>
+      <c r="D175" s="5"/>
+      <c r="E175" s="5"/>
+      <c r="F175" s="5"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="5"/>
+      <c r="B176" s="5"/>
+      <c r="C176" s="5"/>
+      <c r="D176" s="5"/>
+      <c r="E176" s="5"/>
+      <c r="F176" s="5"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="5"/>
+      <c r="B177" s="5"/>
+      <c r="C177" s="5"/>
+      <c r="D177" s="5"/>
+      <c r="E177" s="5"/>
+      <c r="F177" s="5"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>